<commit_message>
Actualizar la ubicacion de cada item del STROBE al manuscrito vigente
Los items apuntaban a frases ya borradas, a Tabla 1/2 (SPM rotula Cuadro I/II) y a un
diseno "ecologico" que el manuscrito ya no declara.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABLAS/STROBE_checklist.xlsx
+++ b/TABLAS/STROBE_checklist.xlsx
@@ -372,7 +372,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Ubicación.en.el.manuscrito</t>
+          <t>Ubicación en el manuscrito</t>
         </is>
       </c>
     </row>
@@ -394,7 +394,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Resumen/Abstract: "Estudio ecológico transversal, análisis secundario"</t>
+          <t>Resumen (Materiales y métodos): "Estudio transversal, análisis secundario de la ENSANUT Continua 2021-2024"</t>
         </is>
       </c>
     </row>
@@ -438,7 +438,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Introducción, párrafos 1-3 (vacío de conocimiento, antecedente INEGI, cascada nacional-estatal ya documentada)</t>
+          <t>Introducción, párrafos 1-4 (vacío de conocimiento, antecedente INEGI, cascada nacional-estatal ya documentada)</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Materiales y métodos &gt; Diseño y fuente de datos (metodología ENSANUT, referencia 12)</t>
+          <t>Materiales y métodos &gt; Diseño y fuente de datos (metodología de la ENSANUT)</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Discusión &gt; Limitaciones (submuestra con presión arterial medida, 43,5% de los entrevistados); Materiales y métodos &gt; Diseño muestral complejo (calibración del ponderador y validación contra el ponderador de tensión arterial de 2023)</t>
+          <t>Discusión &gt; Limitaciones (submuestra con presión arterial medida, 43,5% de los entrevistados); Materiales y métodos &gt; Diseño muestral complejo (calibración del ponderador); Tabla S2, panel A (validación de la calibración contra el ponderador publicado para 2023)</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Resultados &gt; Muestra (ninguna covariable demográfica tuvo dato faltante en la base analítica); Materiales y métodos &gt; Covariables (definición del nivel 'sin escolaridad')</t>
+          <t>Resultados &gt; Muestra y Figura 1 (exclusión de presión arterial no válida, embarazo y ponderador faltante, cada una con su n); Materiales y métodos &gt; Covariables (definición del nivel 'sin escolaridad')</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Materiales y métodos &gt; Reclasificación y validación (sensibilidades a ponderación y matriz de vecindad); Figura S1 (validación cruzada)</t>
+          <t>Materiales y métodos &gt; Reclasificación y validación (sensibilidad a la matriz de vecindad y modelo sin ponderar); Tabla S2, panel B (ponderado frente a sin ponderar); Figura S1 (validación cruzada)</t>
         </is>
       </c>
     </row>
@@ -834,7 +834,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Resultados &gt; Muestra; Tabla 1</t>
+          <t>Resultados &gt; Muestra; Cuadro I</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Resultados &gt; Muestra (0 registros con covariable demográfica faltante); Figura 1 (flujo con el n de cada exclusión)</t>
+          <t>Resultados &gt; Muestra; Figura 1 (flujo con el n de cada exclusión); Cuadro I</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Resultados &gt; Modelos municipales; Figura 2; Tabla 2 (IC95%/credibilidad)</t>
+          <t>Resultados &gt; Modelos municipales; Figura 2; Cuadro II (IC95%/credibilidad)</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Resultados &gt; Reclasificación ESH vs. ACC/AHA; Validación cruzada; Figura 3; Figura S1</t>
+          <t>Resultados &gt; Reclasificación ESH vs. ACC/AHA; Validación cruzada; Figura 3; Figura S1; Tabla S2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Completar el material suplementario: panel B de la Tabla S2, etiquetas y nota de la S4, anios de la S3
El manuscrito citaba el panel B de la Tabla S2 y no existia; la S4 tenia diez etiquetas de
covariable vacias y una nota con cifras viejas; la S3 escribia 2,022 en vez de 2022. El p de
Moran del texto (0,169) pasa a 0,168 como en la S5. El STROBE apunta a lo que si esta.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABLAS/STROBE_checklist.xlsx
+++ b/TABLAS/STROBE_checklist.xlsx
@@ -702,7 +702,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Resultados &gt; Muestra y Figura 1 (exclusión de presión arterial no válida, embarazo y ponderador faltante, cada una con su n); Materiales y métodos &gt; Covariables (definición del nivel 'sin escolaridad')</t>
+          <t>Resultados &gt; Muestra y Figura 1 (exclusión de presión arterial no válida, embarazo y ponderador faltante, cada una con su n); Materiales y métodos &gt; Modelo estadístico (seis registros de control sin pobreza municipal, por tres municipios creados después del marco CONEVAL 2020; Tabla S1)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Resultados &gt; Muestra; Figura 1 (flujo con el n de cada exclusión); Cuadro I</t>
+          <t>Resultados &gt; Muestra; Figura 1 (flujo con el n de cada exclusión); Cuadro I; Materiales y métodos &gt; Modelo estadístico (registros sin pobreza municipal)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corregir el motivo de la pobreza faltante y dejar el STROBE sin remitir a tablas que no existen
Los tres municipios sin pobreza en CONEVAL 2020 figuran como "n.d" (04012, 07125, 29048); solo dos
tienen muestra de control (seis registros). El STROBE ya no atribuye descriptivos ni faltantes al Cuadro I.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TABLAS/STROBE_checklist.xlsx
+++ b/TABLAS/STROBE_checklist.xlsx
@@ -702,7 +702,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Resultados &gt; Muestra y Figura 1 (exclusión de presión arterial no válida, embarazo y ponderador faltante, cada una con su n); Materiales y métodos &gt; Modelo estadístico (seis registros de control sin pobreza municipal, por tres municipios creados después del marco CONEVAL 2020; Tabla S1)</t>
+          <t>Resultados &gt; Muestra y Figura 1 (exclusión de presión arterial no válida, embarazo y ponderador faltante, cada una con su n); Materiales y métodos &gt; Modelo estadístico (seis registros de control de dos municipios sin pobreza publicada por CONEVAL 2020; Tabla S1). Los datos faltantes por covariable no se tabulan en el manuscrito</t>
         </is>
       </c>
     </row>
@@ -834,7 +834,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Resultados &gt; Muestra; Cuadro I</t>
+          <t>Resultados &gt; Muestra; Cuadro I (n por año). Las características sociodemográficas de los participantes no se tabulan en el manuscrito</t>
         </is>
       </c>
     </row>

</xml_diff>